<commit_message>
got analytic vpm working
</commit_message>
<xml_diff>
--- a/output_files/compare_vpm_and_jouk_appellian/appelliean_values_and_error_zeta_clustering=mirrored_cosine_zeta0=(-0.09+0.01j)_D=0.01_surface_offset=1.0e-15.xlsx
+++ b/output_files/compare_vpm_and_jouk_appellian/appelliean_values_and_error_zeta_clustering=mirrored_cosine_zeta0=(-0.09+0.01j)_D=0.01_surface_offset=1.0e-15.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -535,15 +535,25 @@
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
+          <t>appellian_vpm_analytic</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
           <t>appellian_jouk_offset_error</t>
         </is>
       </c>
-      <c r="F10" s="1" t="inlineStr">
+      <c r="G10" s="1" t="inlineStr">
         <is>
           <t>appellian_vpm_error</t>
         </is>
       </c>
-      <c r="G10" s="1" t="inlineStr">
+      <c r="H10" s="1" t="inlineStr">
+        <is>
+          <t>appellian_vpm_analytic_error</t>
+        </is>
+      </c>
+      <c r="I10" s="1" t="inlineStr">
         <is>
           <t>appellian_vpm_vs_offset_error</t>
         </is>
@@ -560,16 +570,22 @@
         <v>18446.34268317429</v>
       </c>
       <c r="D11" t="n">
-        <v>4193563.789408781</v>
+        <v>4193563.789408641</v>
       </c>
       <c r="E11" t="n">
+        <v>4226726.406007651</v>
+      </c>
+      <c r="F11" t="n">
         <v>29.39869180796816</v>
       </c>
-      <c r="F11" t="n">
-        <v>29317.30388960674</v>
-      </c>
       <c r="G11" t="n">
-        <v>22633.84953015055</v>
+        <v>29317.30388960576</v>
+      </c>
+      <c r="H11" t="n">
+        <v>29549.93532655479</v>
+      </c>
+      <c r="I11" t="n">
+        <v>22633.8495301498</v>
       </c>
     </row>
     <row r="12">
@@ -583,16 +599,22 @@
         <v>15440.47870091133</v>
       </c>
       <c r="D12" t="n">
-        <v>37490077.63510653</v>
+        <v>37490077.63519095</v>
       </c>
       <c r="E12" t="n">
+        <v>40419866.19954792</v>
+      </c>
+      <c r="F12" t="n">
         <v>10.05420361020335</v>
       </c>
-      <c r="F12" t="n">
-        <v>267115.8498021711</v>
-      </c>
       <c r="G12" t="n">
-        <v>242703.8557696646</v>
+        <v>267115.8498027728</v>
+      </c>
+      <c r="H12" t="n">
+        <v>287998.3336585069</v>
+      </c>
+      <c r="I12" t="n">
+        <v>242703.8557702113</v>
       </c>
     </row>
     <row r="13">
@@ -606,16 +628,22 @@
         <v>13985.635007918</v>
       </c>
       <c r="D13" t="n">
-        <v>78898788.09078598</v>
+        <v>78898788.09007886</v>
       </c>
       <c r="E13" t="n">
+        <v>111295547.6513574</v>
+      </c>
+      <c r="F13" t="n">
         <v>1.728708066511387</v>
       </c>
-      <c r="F13" t="n">
-        <v>573793.9830722751</v>
-      </c>
       <c r="G13" t="n">
-        <v>564041.6213573229</v>
+        <v>573793.9830671316</v>
+      </c>
+      <c r="H13" t="n">
+        <v>809441.5238362425</v>
+      </c>
+      <c r="I13" t="n">
+        <v>564041.6213522669</v>
       </c>
     </row>
     <row r="14">
@@ -629,16 +657,22 @@
         <v>13695.12805008676</v>
       </c>
       <c r="D14" t="n">
-        <v>34304566.05385566</v>
+        <v>34304566.05387905</v>
       </c>
       <c r="E14" t="n">
+        <v>108064310.2196071</v>
+      </c>
+      <c r="F14" t="n">
         <v>0.2352001632288192</v>
       </c>
-      <c r="F14" t="n">
-        <v>250976.5165791307</v>
-      </c>
       <c r="G14" t="n">
-        <v>250387.369876314</v>
+        <v>250976.5165793019</v>
+      </c>
+      <c r="H14" t="n">
+        <v>790827.0892355733</v>
+      </c>
+      <c r="I14" t="n">
+        <v>250387.3698764848</v>
       </c>
     </row>
     <row r="15">
@@ -652,16 +686,22 @@
         <v>13630.07190490942</v>
       </c>
       <c r="D15" t="n">
-        <v>9101734.506155293</v>
+        <v>9101734.506085351</v>
       </c>
       <c r="E15" t="n">
+        <v>107449312.5139183</v>
+      </c>
+      <c r="F15" t="n">
         <v>0.1027760182874937</v>
       </c>
-      <c r="F15" t="n">
-        <v>66608.23286383237</v>
-      </c>
       <c r="G15" t="n">
-        <v>66676.86346523922</v>
+        <v>66608.23286331975</v>
+      </c>
+      <c r="H15" t="n">
+        <v>787415.1439969788</v>
+      </c>
+      <c r="I15" t="n">
+        <v>66676.86346472608</v>
       </c>
     </row>
     <row r="16">
@@ -675,16 +715,22 @@
         <v>13615.87290332567</v>
       </c>
       <c r="D16" t="n">
-        <v>2311738.307786231</v>
+        <v>2311738.282046879</v>
       </c>
       <c r="E16" t="n">
+        <v>108671277.6205768</v>
+      </c>
+      <c r="F16" t="n">
         <v>0.1852035248434549</v>
       </c>
-      <c r="F16" t="n">
-        <v>16846.81570060381</v>
-      </c>
       <c r="G16" t="n">
-        <v>16878.26003664877</v>
+        <v>16846.81551191461</v>
+      </c>
+      <c r="H16" t="n">
+        <v>796543.8534942358</v>
+      </c>
+      <c r="I16" t="n">
+        <v>16878.25984760946</v>
       </c>
     </row>
     <row r="17">
@@ -698,108 +744,22 @@
         <v>13612.33595090774</v>
       </c>
       <c r="D17" t="n">
-        <v>589060.5836424412</v>
+        <v>589060.5834069725</v>
       </c>
       <c r="E17" t="n">
+        <v>109732673.811397</v>
+      </c>
+      <c r="F17" t="n">
         <v>0.2057561586903014</v>
       </c>
-      <c r="F17" t="n">
-        <v>4218.498730366548</v>
-      </c>
       <c r="G17" t="n">
-        <v>4227.40262778454</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>2560</v>
-      </c>
-      <c r="B18" t="n">
-        <v>13640.21820451814</v>
-      </c>
-      <c r="C18" t="n">
-        <v>13611.4523760223</v>
-      </c>
-      <c r="D18" t="n">
-        <v>151231.6226610602</v>
-      </c>
-      <c r="E18" t="n">
-        <v>0.2108897971024366</v>
-      </c>
-      <c r="F18" t="n">
-        <v>1008.718499906158</v>
-      </c>
-      <c r="G18" t="n">
-        <v>1011.061615492754</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>5120</v>
-      </c>
-      <c r="B19" t="n">
-        <v>13640.17227611977</v>
-      </c>
-      <c r="C19" t="n">
-        <v>13611.23152375479</v>
-      </c>
-      <c r="D19" t="n">
-        <v>45400.34864611717</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0.21217292405937</v>
-      </c>
-      <c r="F19" t="n">
-        <v>232.8429269592206</v>
-      </c>
-      <c r="G19" t="n">
-        <v>233.5506310864151</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>10240</v>
-      </c>
-      <c r="B20" t="n">
-        <v>13640.16079401688</v>
-      </c>
-      <c r="C20" t="n">
-        <v>13611.17631327849</v>
-      </c>
-      <c r="D20" t="n">
-        <v>15982.66729836096</v>
-      </c>
-      <c r="E20" t="n">
-        <v>0.2124936881323064</v>
-      </c>
-      <c r="F20" t="n">
-        <v>17.17359890193967</v>
-      </c>
-      <c r="G20" t="n">
-        <v>17.42311561102139</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>20480</v>
-      </c>
-      <c r="B21" t="n">
-        <v>13640.15792349101</v>
-      </c>
-      <c r="C21" t="n">
-        <v>13611.16251082143</v>
-      </c>
-      <c r="D21" t="n">
-        <v>8320.729362415521</v>
-      </c>
-      <c r="E21" t="n">
-        <v>0.2125738780461419</v>
-      </c>
-      <c r="F21" t="n">
-        <v>38.99829159539567</v>
-      </c>
-      <c r="G21" t="n">
-        <v>38.86834165854532</v>
+        <v>4218.498728640288</v>
+      </c>
+      <c r="H17" t="n">
+        <v>804368.0389307614</v>
+      </c>
+      <c r="I17" t="n">
+        <v>4227.402626054721</v>
       </c>
     </row>
   </sheetData>

</xml_diff>